<commit_message>
Sheet template: theme soft limit 80 -> 110, row-layout wording
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dk24v8pFVzWVUg3pzjuvx8
</commit_message>
<xml_diff>
--- a/sheet-template/Topic Marketplace Rooms.xlsx
+++ b/sheet-template/Topic Marketplace Rooms.xlsx
@@ -761,7 +761,7 @@
   </sheetData>
   <conditionalFormatting sqref="B2:B21">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>LEN(B2)&gt;80</formula>
+      <formula>LEN(B2)&gt;110</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C21">
@@ -771,7 +771,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D21">
     <cfRule type="expression" priority="3" dxfId="0">
-      <formula>LEN(D2)&gt;80</formula>
+      <formula>LEN(D2)&gt;110</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E21">
@@ -785,14 +785,14 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">
-    <dataValidation sqref="B2:B21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Long for the projector" error="Over 80 characters. It will still show, but text shrinks for every room. Shorten if you can." promptTitle="Up to ~80 characters" prompt="Keep it short; it's read from the back of the room." type="custom" errorStyle="warning">
-      <formula1>LEN(B2)&lt;=80</formula1>
+    <dataValidation sqref="B2:B21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Long for the projector" error="Over 110 characters. It will still show, but text shrinks for every room. Shorten if you can." promptTitle="Up to ~110 characters" prompt="Keep it short; it's read from the back of the room." type="custom" errorStyle="warning">
+      <formula1>LEN(B2)&lt;=110</formula1>
     </dataValidation>
     <dataValidation sqref="C2:C21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Long for the projector" error="Over 140 characters. It will still show, but text shrinks for every room. Shorten if you can." promptTitle="Up to ~140 characters" prompt="Context: one line per bullet (Ctrl+Enter or Alt+Enter for a new line)." type="custom" errorStyle="warning">
       <formula1>LEN(C2)&lt;=140</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Long for the projector" error="Over 80 characters. It will still show, but text shrinks for every room. Shorten if you can." promptTitle="Up to ~80 characters" prompt="Keep it short; it's read from the back of the room." type="custom" errorStyle="warning">
-      <formula1>LEN(D2)&lt;=80</formula1>
+    <dataValidation sqref="D2:D21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Long for the projector" error="Over 110 characters. It will still show, but text shrinks for every room. Shorten if you can." promptTitle="Up to ~110 characters" prompt="Keep it short; it's read from the back of the room." type="custom" errorStyle="warning">
+      <formula1>LEN(D2)&lt;=110</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Long for the projector" error="Over 140 characters. It will still show, but text shrinks for every room. Shorten if you can." promptTitle="Up to ~140 characters" prompt="Context: one line per bullet (Ctrl+Enter or Alt+Enter for a new line)." type="custom" errorStyle="warning">
       <formula1>LEN(E2)&lt;=140</formula1>
@@ -889,7 +889,7 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>- Row order is display order. Reorder rooms by moving rows; the grid sizes itself to the room count (12 -&gt; 4x3, 13 -&gt; 5x3).</t>
+          <t>- Row order is display order. Reorder rooms by moving rows; the grid sizes itself to the room count (12 -&gt; 4/4/4, 13 -&gt; 5/4/4).</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Limits: themes 80, context 140, note 60 characters.</t>
+          <t xml:space="preserve">  Limits: themes 110, context 140, note 60 characters.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sheet template: Group column, split-room naming, updated instructions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dk24v8pFVzWVUg3pzjuvx8
</commit_message>
<xml_diff>
--- a/sheet-template/Topic Marketplace Rooms.xlsx
+++ b/sheet-template/Topic Marketplace Rooms.xlsx
@@ -503,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -512,6 +512,7 @@
     <col width="42" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
     <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -545,11 +546,16 @@
           <t>Note</t>
         </is>
       </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Canal Room - 1</t>
+          <t>Canal - 1</t>
         </is>
       </c>
       <c r="B2" s="6" t="n"/>
@@ -557,11 +563,16 @@
       <c r="D2" s="6" t="n"/>
       <c r="E2" s="6" t="n"/>
       <c r="F2" s="6" t="n"/>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Ballroom</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Canal Room - 2</t>
+          <t>Canal - 2</t>
         </is>
       </c>
       <c r="B3" s="6" t="n"/>
@@ -569,11 +580,16 @@
       <c r="D3" s="6" t="n"/>
       <c r="E3" s="6" t="n"/>
       <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Ballroom</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Millpond Room - 1</t>
+          <t>Millpond - 1</t>
         </is>
       </c>
       <c r="B4" s="6" t="n"/>
@@ -581,11 +597,16 @@
       <c r="D4" s="6" t="n"/>
       <c r="E4" s="6" t="n"/>
       <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Ballroom</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Millpond Room - 2</t>
+          <t>Millpond - 2</t>
         </is>
       </c>
       <c r="B5" s="6" t="n"/>
@@ -593,11 +614,16 @@
       <c r="D5" s="6" t="n"/>
       <c r="E5" s="6" t="n"/>
       <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Ballroom</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Great Falls Room - 1</t>
+          <t>Great Falls - 1</t>
         </is>
       </c>
       <c r="B6" s="6" t="n"/>
@@ -605,11 +631,16 @@
       <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Ballroom</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Great Falls Room - 2</t>
+          <t>Great Falls - 2</t>
         </is>
       </c>
       <c r="B7" s="6" t="n"/>
@@ -617,11 +648,16 @@
       <c r="D7" s="6" t="n"/>
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Ballroom</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Ballroom Rotunda</t>
+          <t>Rotunda</t>
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
@@ -629,6 +665,11 @@
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Ballroom</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -641,6 +682,11 @@
       <c r="D9" s="6" t="n"/>
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Meeting rooms</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -653,6 +699,11 @@
       <c r="D10" s="6" t="n"/>
       <c r="E10" s="6" t="n"/>
       <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Meeting rooms</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -665,6 +716,11 @@
       <c r="D11" s="6" t="n"/>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Meeting rooms</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -677,6 +733,11 @@
       <c r="D12" s="6" t="n"/>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Meeting rooms</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -689,6 +750,11 @@
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Meeting rooms</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -701,6 +767,11 @@
       <c r="D14" s="6" t="n"/>
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Meeting rooms</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="5" t="n"/>
@@ -709,6 +780,7 @@
       <c r="D15" s="6" t="n"/>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="5" t="n"/>
@@ -717,6 +789,7 @@
       <c r="D16" s="6" t="n"/>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="5" t="n"/>
@@ -725,6 +798,7 @@
       <c r="D17" s="6" t="n"/>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="5" t="n"/>
@@ -733,6 +807,7 @@
       <c r="D18" s="6" t="n"/>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="5" t="n"/>
@@ -741,6 +816,7 @@
       <c r="D19" s="6" t="n"/>
       <c r="E19" s="6" t="n"/>
       <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
     </row>
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="5" t="n"/>
@@ -749,6 +825,7 @@
       <c r="D20" s="6" t="n"/>
       <c r="E20" s="6" t="n"/>
       <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
     </row>
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="5" t="n"/>
@@ -757,6 +834,7 @@
       <c r="D21" s="6" t="n"/>
       <c r="E21" s="6" t="n"/>
       <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B21">
@@ -811,7 +889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -827,7 +905,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>The display page reads the 'Display' tab every ~3 seconds and shows one card per row, in row order.</t>
+          <t>The display page reads the 'Display' tab every ~3 seconds and shows one card per room, in row order.</t>
         </is>
       </c>
     </row>
@@ -882,71 +960,92 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>- Keep the tab named 'Display' and keep the header row and column order (Room, AM theme, AM context, PM theme, PM context, Note).</t>
+          <t>- Keep the tab named 'Display' and keep the header row and column order (Room, AM theme, AM context, PM theme, PM context, Note, Group).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>- Row order is display order. Reorder rooms by moving rows; the grid sizes itself to the room count (12 -&gt; 4/4/4, 13 -&gt; 5/4/4).</t>
+          <t>- Row order is display order. Reorder rooms by moving rows; the layout picks whatever row arrangement gives the largest text.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>- A row with a blank Room is skipped, so you can leave spare rows at the bottom.</t>
+          <t>- Two conversations in one room: name the rows '&lt;Room&gt; - 1' and '&lt;Room&gt; - 2' (e.g. Canal - 1, Canal - 2). They share one card, split in half.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr"/>
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>- Group: rooms with the same Group (e.g. Ballroom, Meeting rooms) sit together under that label. Leave Group blank everywhere for no grouping.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>Typing on the day</t>
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>- Keep room names short (e.g. Canal - 1) so each name fits on one line of its card header.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>- Theme: the topic title. Context: optional supporting lines; each line in the cell becomes its own line on the card (Ctrl+Enter or Alt+Enter).</t>
+          <t>- A row with a blank Room is skipped, so you can leave spare rows at the bottom.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>- Blank theme shows 'Topic coming soon', so unfilled rooms look intentional.</t>
-        </is>
-      </c>
+      <c r="A17" s="8" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>- Note: if both themes are blank, the Note fills the card (e.g. 'Reset Room: open all day', 'Not in use'). Otherwise it shows as a small line under the topics.</t>
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Typing on the day</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>- Red cell = over the soft length limit. It still displays, but every card's text shrinks to fit, so shorten if you can.</t>
+          <t>- Theme: the topic title. Context: optional supporting lines; each line in the cell becomes its own line on the card (Ctrl+Enter or Alt+Enter).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Limits: themes 110, context 140, note 60 characters.</t>
+          <t>- Blank theme shows 'Topic coming soon', so unfilled rooms look intentional.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>- Note: if both themes are blank, the Note fills the card (e.g. 'Reset Room: open all day', 'Not in use'). Otherwise it shows as a small line under the topics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>- Red cell = over the soft length limit. It still displays, but that card's text shrinks to fit, so shorten if you can.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Limits: themes 110, context 140, note 60 characters. Each card sizes its own text; only the wordiest cards shrink.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>- The projector laptop never opens this Sheet; type from a second device.</t>
         </is>

</xml_diff>

<commit_message>
White header with TFG logo and QR code, phone layout, tap-for-details
- Header: smaller title, TFG logo, QR code to the page in place of the clock
- Projector shows themes only; context moves to a details sheet opened by tapping a card
- Phones and portrait screens get a scrolling, grouped list with a bottom-sheet detail view
- Split-room halves size to their content, so the afternoon slot no longer sits on the card's bottom edge
- make_assets.py builds logo.png and qr.svg; context soft limit 140 -> 300 (tap-only now)
- Drop the prototype's demo edit/reorder mode (the Sheet is the editor now)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dk24v8pFVzWVUg3pzjuvx8
</commit_message>
<xml_diff>
--- a/sheet-template/Topic Marketplace Rooms.xlsx
+++ b/sheet-template/Topic Marketplace Rooms.xlsx
@@ -844,7 +844,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C21">
     <cfRule type="expression" priority="2" dxfId="0">
-      <formula>LEN(C2)&gt;140</formula>
+      <formula>LEN(C2)&gt;300</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D21">
@@ -854,7 +854,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E21">
     <cfRule type="expression" priority="4" dxfId="0">
-      <formula>LEN(E2)&gt;140</formula>
+      <formula>LEN(E2)&gt;300</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F21">
@@ -866,14 +866,14 @@
     <dataValidation sqref="B2:B21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Long for the projector" error="Over 110 characters. It will still show, but text shrinks for every room. Shorten if you can." promptTitle="Up to ~110 characters" prompt="Keep it short; it's read from the back of the room." type="custom" errorStyle="warning">
       <formula1>LEN(B2)&lt;=110</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Long for the projector" error="Over 140 characters. It will still show, but text shrinks for every room. Shorten if you can." promptTitle="Up to ~140 characters" prompt="Context: one line per bullet (Ctrl+Enter or Alt+Enter for a new line)." type="custom" errorStyle="warning">
-      <formula1>LEN(C2)&lt;=140</formula1>
+    <dataValidation sqref="C2:C21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Long for the projector" error="Over 300 characters. It will still show, but text shrinks for every room. Shorten if you can." promptTitle="Up to ~300 characters" prompt="Context: shows when someone taps the card, not on the projector. One line per bullet (Ctrl+Enter or Alt+Enter)." type="custom" errorStyle="warning">
+      <formula1>LEN(C2)&lt;=300</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Long for the projector" error="Over 110 characters. It will still show, but text shrinks for every room. Shorten if you can." promptTitle="Up to ~110 characters" prompt="Keep it short; it's read from the back of the room." type="custom" errorStyle="warning">
       <formula1>LEN(D2)&lt;=110</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Long for the projector" error="Over 140 characters. It will still show, but text shrinks for every room. Shorten if you can." promptTitle="Up to ~140 characters" prompt="Context: one line per bullet (Ctrl+Enter or Alt+Enter for a new line)." type="custom" errorStyle="warning">
-      <formula1>LEN(E2)&lt;=140</formula1>
+    <dataValidation sqref="E2:E21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Long for the projector" error="Over 300 characters. It will still show, but text shrinks for every room. Shorten if you can." promptTitle="Up to ~300 characters" prompt="Context: shows when someone taps the card, not on the projector. One line per bullet (Ctrl+Enter or Alt+Enter)." type="custom" errorStyle="warning">
+      <formula1>LEN(E2)&lt;=300</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Long for the projector" error="Over 60 characters. It will still show, but text shrinks for every room. Shorten if you can." promptTitle="Up to ~60 characters" prompt="Fills the whole card if both themes are blank (e.g. Reset Room: open all day)." type="custom" errorStyle="warning">
       <formula1>LEN(F2)&lt;=60</formula1>
@@ -905,7 +905,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>The display page reads the 'Display' tab every ~3 seconds and shows one card per room, in row order.</t>
+          <t>The display page reads the 'Display' tab every ~3 seconds and shows one card per room, in row order. Attendees can open the same page on their phones via the QR code.</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>- Theme: the topic title. Context: optional supporting lines; each line in the cell becomes its own line on the card (Ctrl+Enter or Alt+Enter).</t>
+          <t>- Theme: the topic title; this is what the projector shows. Context: optional supporting lines, shown only when someone taps the card on a phone or laptop (one line per bullet: Ctrl+Enter or Alt+Enter). Cards with context get a small More tag.</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Limits: themes 110, context 140, note 60 characters. Each card sizes its own text; only the wordiest cards shrink.</t>
+          <t xml:space="preserve">  Limits: themes 110, note 60 characters (projector); context 300 (tap-to-view only). Each card sizes its own text; only the wordiest cards shrink.</t>
         </is>
       </c>
     </row>

</xml_diff>